<commit_message>
Q4S-Timesheet: duidelijk onderscheid normale uren (zwarte band met uitleg) en overuren (oranje blok met eigen dagkoppen, getinte invulvakken, oranje totaal) in Excel en dashboard-voorbeeld
</commit_message>
<xml_diff>
--- a/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
+++ b/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
     <numFmt numFmtId="165" formatCode="DD-MM"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,14 +68,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="006B6B70"/>
-      <sz val="8"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <color rgb="006B6B70"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -95,6 +95,18 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C2410C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C2410C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="001C1C1E"/>
       <sz val="8"/>
     </font>
@@ -105,7 +117,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -125,6 +137,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FAFAFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C2410C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -155,6 +177,12 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
       <bottom style="thin">
         <color rgb="001C1C1E"/>
       </bottom>
@@ -173,12 +201,6 @@
       <top style="thin">
         <color rgb="001C1C1E"/>
       </top>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom/>
     </border>
     <border>
@@ -229,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -262,21 +284,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -291,10 +316,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -303,22 +328,50 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -879,264 +932,280 @@
       <c r="P8" s="11" t="n"/>
       <c r="Q8" s="11" t="n"/>
     </row>
-    <row r="9" ht="6" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>NORMAL HOURS — regular hours per day. Hours above the regular schedule go in the orange OVERTIME block below.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Client / Proj. no.</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Hour code</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="15">
         <f>IF(Q2="","",Q2+0)</f>
         <v/>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="15">
         <f>IF(Q2="","",Q2+1)</f>
         <v/>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="15">
         <f>IF(Q2="","",Q2+2)</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="15">
         <f>IF(Q2="","",Q2+3)</f>
         <v/>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="15">
         <f>IF(Q2="","",Q2+4)</f>
         <v/>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="15">
         <f>IF(Q2="","",Q2+5)</f>
         <v/>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="15">
         <f>IF(Q2="","",Q2+6)</f>
         <v/>
       </c>
-      <c r="L10" s="14" t="inlineStr">
+      <c r="L10" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="N10" s="15" t="inlineStr">
+      <c r="N10" s="17" t="inlineStr">
         <is>
           <t>Kilometres</t>
         </is>
       </c>
-      <c r="O10" s="16" t="n"/>
-      <c r="P10" s="16" t="n"/>
-      <c r="Q10" s="16" t="n"/>
+      <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="13" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="I11" s="15" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="J11" s="15" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="K11" s="15" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="N11" s="18" t="inlineStr"/>
-      <c r="O11" s="18" t="inlineStr">
+      <c r="L11" s="18" t="n"/>
+      <c r="N11" s="19" t="inlineStr"/>
+      <c r="O11" s="19" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="P11" s="18" t="inlineStr">
+      <c r="P11" s="19" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="Q11" s="18" t="inlineStr">
+      <c r="Q11" s="19" t="inlineStr">
         <is>
           <t>Km</t>
         </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="22">
+      <c r="B12" s="20" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="21" t="n"/>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="22" t="n"/>
+      <c r="L12" s="23">
         <f>IF(SUM(E12:K12)=0,"",SUM(E12:K12))</f>
         <v/>
       </c>
-      <c r="N12" s="15" t="inlineStr">
+      <c r="N12" s="17" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="O12" s="23" t="n"/>
-      <c r="P12" s="23" t="n"/>
-      <c r="Q12" s="24" t="n"/>
+      <c r="O12" s="24" t="n"/>
+      <c r="P12" s="24" t="n"/>
+      <c r="Q12" s="25" t="n"/>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="21" t="n"/>
-      <c r="K13" s="21" t="n"/>
-      <c r="L13" s="22">
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="21" t="n"/>
+      <c r="J13" s="22" t="n"/>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="23">
         <f>IF(SUM(E13:K13)=0,"",SUM(E13:K13))</f>
         <v/>
       </c>
-      <c r="N13" s="13">
+      <c r="N13" s="15">
         <f>E10</f>
         <v/>
       </c>
-      <c r="O13" s="23" t="n"/>
-      <c r="P13" s="23" t="n"/>
-      <c r="Q13" s="24" t="n"/>
+      <c r="O13" s="24" t="n"/>
+      <c r="P13" s="24" t="n"/>
+      <c r="Q13" s="25" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="20" t="n"/>
-      <c r="I14" s="20" t="n"/>
-      <c r="J14" s="21" t="n"/>
-      <c r="K14" s="21" t="n"/>
-      <c r="L14" s="22">
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
+      <c r="I14" s="21" t="n"/>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="23">
         <f>IF(SUM(E14:K14)=0,"",SUM(E14:K14))</f>
         <v/>
       </c>
-      <c r="N14" s="17" t="n"/>
-      <c r="O14" s="23" t="n"/>
-      <c r="P14" s="23" t="n"/>
-      <c r="Q14" s="24" t="n"/>
+      <c r="N14" s="18" t="n"/>
+      <c r="O14" s="24" t="n"/>
+      <c r="P14" s="24" t="n"/>
+      <c r="Q14" s="25" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="21" t="n"/>
-      <c r="K15" s="21" t="n"/>
-      <c r="L15" s="22">
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="22" t="n"/>
+      <c r="L15" s="23">
         <f>IF(SUM(E15:K15)=0,"",SUM(E15:K15))</f>
         <v/>
       </c>
-      <c r="N15" s="17" t="n"/>
-      <c r="O15" s="23" t="n"/>
-      <c r="P15" s="23" t="n"/>
-      <c r="Q15" s="24" t="n"/>
+      <c r="N15" s="18" t="n"/>
+      <c r="O15" s="24" t="n"/>
+      <c r="P15" s="24" t="n"/>
+      <c r="Q15" s="25" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="20" t="n"/>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="n"/>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="20" t="n"/>
-      <c r="I16" s="20" t="n"/>
-      <c r="J16" s="21" t="n"/>
-      <c r="K16" s="21" t="n"/>
-      <c r="L16" s="22">
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="21" t="n"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="21" t="n"/>
+      <c r="I16" s="21" t="n"/>
+      <c r="J16" s="22" t="n"/>
+      <c r="K16" s="22" t="n"/>
+      <c r="L16" s="23">
         <f>IF(SUM(E16:K16)=0,"",SUM(E16:K16))</f>
         <v/>
       </c>
-      <c r="N16" s="15" t="inlineStr">
+      <c r="N16" s="17" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="O16" s="23" t="n"/>
-      <c r="P16" s="23" t="n"/>
-      <c r="Q16" s="24" t="n"/>
+      <c r="O16" s="24" t="n"/>
+      <c r="P16" s="24" t="n"/>
+      <c r="Q16" s="25" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="E17" s="20" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="20" t="n"/>
-      <c r="H17" s="20" t="n"/>
-      <c r="I17" s="20" t="n"/>
-      <c r="J17" s="21" t="n"/>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="22">
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="22" t="n"/>
+      <c r="L17" s="23">
         <f>IF(SUM(E17:K17)=0,"",SUM(E17:K17))</f>
         <v/>
       </c>
-      <c r="N17" s="13">
+      <c r="N17" s="15">
         <f>F10</f>
         <v/>
       </c>
-      <c r="O17" s="23" t="n"/>
-      <c r="P17" s="23" t="n"/>
-      <c r="Q17" s="24" t="n"/>
+      <c r="O17" s="24" t="n"/>
+      <c r="P17" s="24" t="n"/>
+      <c r="Q17" s="25" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>Hours worked</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Total normal hours</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
       <c r="E18" s="7">
         <f>SUM(E12:E17)</f>
         <v/>
@@ -1165,174 +1234,206 @@
         <f>SUM(K12:K17)</f>
         <v/>
       </c>
-      <c r="L18" s="26">
+      <c r="L18" s="27">
         <f>SUM(E18:K18)</f>
         <v/>
       </c>
-      <c r="N18" s="17" t="n"/>
-      <c r="O18" s="23" t="n"/>
-      <c r="P18" s="23" t="n"/>
-      <c r="Q18" s="24" t="n"/>
+      <c r="N18" s="18" t="n"/>
+      <c r="O18" s="24" t="n"/>
+      <c r="P18" s="24" t="n"/>
+      <c r="Q18" s="25" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="N19" s="17" t="n"/>
-      <c r="O19" s="23" t="n"/>
-      <c r="P19" s="23" t="n"/>
-      <c r="Q19" s="24" t="n"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Overtime</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
-      <c r="H20" s="11" t="n"/>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11" t="n"/>
-      <c r="L20" s="11" t="n"/>
-      <c r="N20" s="15" t="inlineStr">
+      <c r="N19" s="18" t="n"/>
+      <c r="O19" s="24" t="n"/>
+      <c r="P19" s="24" t="n"/>
+      <c r="Q19" s="25" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>OVERTIME (extra hrs)</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="n"/>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>Mo</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>Tu</t>
+        </is>
+      </c>
+      <c r="G20" s="30" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="O20" s="23" t="n"/>
-      <c r="P20" s="23" t="n"/>
-      <c r="Q20" s="24" t="n"/>
+      <c r="H20" s="30" t="inlineStr">
+        <is>
+          <t>Th</t>
+        </is>
+      </c>
+      <c r="I20" s="30" t="inlineStr">
+        <is>
+          <t>Fr</t>
+        </is>
+      </c>
+      <c r="J20" s="30" t="inlineStr">
+        <is>
+          <t>Sa</t>
+        </is>
+      </c>
+      <c r="K20" s="30" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
+      </c>
+      <c r="L20" s="31" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>We</t>
+        </is>
+      </c>
+      <c r="O20" s="24" t="n"/>
+      <c r="P20" s="24" t="n"/>
+      <c r="Q20" s="25" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="n"/>
-      <c r="F21" s="20" t="n"/>
-      <c r="G21" s="20" t="n"/>
-      <c r="H21" s="20" t="n"/>
-      <c r="I21" s="20" t="n"/>
-      <c r="J21" s="21" t="n"/>
-      <c r="K21" s="21" t="n"/>
-      <c r="L21" s="22">
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="n"/>
+      <c r="I21" s="33" t="n"/>
+      <c r="J21" s="33" t="n"/>
+      <c r="K21" s="33" t="n"/>
+      <c r="L21" s="34">
         <f>IF(SUM(E21:K21)=0,"",SUM(E21:K21))</f>
         <v/>
       </c>
-      <c r="N21" s="13">
+      <c r="N21" s="15">
         <f>G10</f>
         <v/>
       </c>
-      <c r="O21" s="23" t="n"/>
-      <c r="P21" s="23" t="n"/>
-      <c r="Q21" s="24" t="n"/>
+      <c r="O21" s="24" t="n"/>
+      <c r="P21" s="24" t="n"/>
+      <c r="Q21" s="25" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="20" t="n"/>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="20" t="n"/>
-      <c r="J22" s="21" t="n"/>
-      <c r="K22" s="21" t="n"/>
-      <c r="L22" s="22">
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n"/>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="33" t="n"/>
+      <c r="L22" s="34">
         <f>IF(SUM(E22:K22)=0,"",SUM(E22:K22))</f>
         <v/>
       </c>
-      <c r="N22" s="17" t="n"/>
-      <c r="O22" s="23" t="n"/>
-      <c r="P22" s="23" t="n"/>
-      <c r="Q22" s="24" t="n"/>
+      <c r="N22" s="18" t="n"/>
+      <c r="O22" s="24" t="n"/>
+      <c r="P22" s="24" t="n"/>
+      <c r="Q22" s="25" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="20" t="n"/>
-      <c r="H23" s="20" t="n"/>
-      <c r="I23" s="20" t="n"/>
-      <c r="J23" s="21" t="n"/>
-      <c r="K23" s="21" t="n"/>
-      <c r="L23" s="22">
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="n"/>
+      <c r="I23" s="33" t="n"/>
+      <c r="J23" s="33" t="n"/>
+      <c r="K23" s="33" t="n"/>
+      <c r="L23" s="34">
         <f>IF(SUM(E23:K23)=0,"",SUM(E23:K23))</f>
         <v/>
       </c>
-      <c r="N23" s="17" t="n"/>
-      <c r="O23" s="23" t="n"/>
-      <c r="P23" s="23" t="n"/>
-      <c r="Q23" s="24" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="24" t="n"/>
+      <c r="P23" s="24" t="n"/>
+      <c r="Q23" s="25" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="25" t="inlineStr">
-        <is>
-          <t>Overtime hrs</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="n"/>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="7">
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>Total overtime</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="36">
         <f>SUM(E21:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="36">
         <f>SUM(F21:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="36">
         <f>SUM(G21:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="36">
         <f>SUM(H21:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="36">
         <f>SUM(I21:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="7">
+      <c r="J24" s="36">
         <f>SUM(J21:J23)</f>
         <v/>
       </c>
-      <c r="K24" s="7">
+      <c r="K24" s="36">
         <f>SUM(K21:K23)</f>
         <v/>
       </c>
-      <c r="L24" s="26">
+      <c r="L24" s="37">
         <f>SUM(E24:K24)</f>
         <v/>
       </c>
-      <c r="N24" s="15" t="inlineStr">
+      <c r="N24" s="17" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="O24" s="23" t="n"/>
-      <c r="P24" s="23" t="n"/>
-      <c r="Q24" s="24" t="n"/>
+      <c r="O24" s="24" t="n"/>
+      <c r="P24" s="24" t="n"/>
+      <c r="Q24" s="25" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="N25" s="13">
+      <c r="N25" s="15">
         <f>H10</f>
         <v/>
       </c>
-      <c r="O25" s="23" t="n"/>
-      <c r="P25" s="23" t="n"/>
-      <c r="Q25" s="24" t="n"/>
+      <c r="O25" s="24" t="n"/>
+      <c r="P25" s="24" t="n"/>
+      <c r="Q25" s="25" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="38" t="inlineStr">
         <is>
           <t>Description of work</t>
         </is>
@@ -1346,467 +1447,467 @@
       <c r="J26" s="11" t="n"/>
       <c r="K26" s="11" t="n"/>
       <c r="L26" s="11" t="n"/>
-      <c r="N26" s="17" t="n"/>
-      <c r="O26" s="23" t="n"/>
-      <c r="P26" s="23" t="n"/>
-      <c r="Q26" s="24" t="n"/>
+      <c r="N26" s="18" t="n"/>
+      <c r="O26" s="24" t="n"/>
+      <c r="P26" s="24" t="n"/>
+      <c r="Q26" s="25" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="C27" s="28" t="n"/>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
-      <c r="G27" s="17" t="n"/>
-      <c r="H27" s="17" t="n"/>
-      <c r="I27" s="17" t="n"/>
-      <c r="J27" s="17" t="n"/>
-      <c r="K27" s="17" t="n"/>
-      <c r="L27" s="17" t="n"/>
-      <c r="N27" s="17" t="n"/>
-      <c r="O27" s="23" t="n"/>
-      <c r="P27" s="23" t="n"/>
-      <c r="Q27" s="24" t="n"/>
+      <c r="C27" s="39" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="N27" s="18" t="n"/>
+      <c r="O27" s="24" t="n"/>
+      <c r="P27" s="24" t="n"/>
+      <c r="Q27" s="25" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="13">
+      <c r="B28" s="15">
         <f>E10</f>
         <v/>
       </c>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="17" t="n"/>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
-      <c r="G28" s="17" t="n"/>
-      <c r="H28" s="17" t="n"/>
-      <c r="I28" s="17" t="n"/>
-      <c r="J28" s="17" t="n"/>
-      <c r="K28" s="17" t="n"/>
-      <c r="L28" s="17" t="n"/>
-      <c r="N28" s="15" t="inlineStr">
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="18" t="n"/>
+      <c r="F28" s="18" t="n"/>
+      <c r="G28" s="18" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="18" t="n"/>
+      <c r="J28" s="18" t="n"/>
+      <c r="K28" s="18" t="n"/>
+      <c r="L28" s="18" t="n"/>
+      <c r="N28" s="17" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="O28" s="23" t="n"/>
-      <c r="P28" s="23" t="n"/>
-      <c r="Q28" s="24" t="n"/>
+      <c r="O28" s="24" t="n"/>
+      <c r="P28" s="24" t="n"/>
+      <c r="Q28" s="25" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="C29" s="28" t="n"/>
-      <c r="D29" s="17" t="n"/>
-      <c r="E29" s="17" t="n"/>
-      <c r="F29" s="17" t="n"/>
-      <c r="G29" s="17" t="n"/>
-      <c r="H29" s="17" t="n"/>
-      <c r="I29" s="17" t="n"/>
-      <c r="J29" s="17" t="n"/>
-      <c r="K29" s="17" t="n"/>
-      <c r="L29" s="17" t="n"/>
-      <c r="N29" s="13">
+      <c r="C29" s="39" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
+      <c r="L29" s="18" t="n"/>
+      <c r="N29" s="15">
         <f>I10</f>
         <v/>
       </c>
-      <c r="O29" s="23" t="n"/>
-      <c r="P29" s="23" t="n"/>
-      <c r="Q29" s="24" t="n"/>
+      <c r="O29" s="24" t="n"/>
+      <c r="P29" s="24" t="n"/>
+      <c r="Q29" s="25" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="13">
+      <c r="B30" s="15">
         <f>F10</f>
         <v/>
       </c>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-      <c r="K30" s="17" t="n"/>
-      <c r="L30" s="17" t="n"/>
-      <c r="N30" s="17" t="n"/>
-      <c r="O30" s="23" t="n"/>
-      <c r="P30" s="23" t="n"/>
-      <c r="Q30" s="24" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="24" t="n"/>
+      <c r="P30" s="24" t="n"/>
+      <c r="Q30" s="25" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="17" t="n"/>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
-      <c r="G31" s="17" t="n"/>
-      <c r="H31" s="17" t="n"/>
-      <c r="I31" s="17" t="n"/>
-      <c r="J31" s="17" t="n"/>
-      <c r="K31" s="17" t="n"/>
-      <c r="L31" s="17" t="n"/>
-      <c r="N31" s="17" t="n"/>
-      <c r="O31" s="23" t="n"/>
-      <c r="P31" s="23" t="n"/>
-      <c r="Q31" s="24" t="n"/>
+      <c r="C31" s="39" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="18" t="n"/>
+      <c r="K31" s="18" t="n"/>
+      <c r="L31" s="18" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="24" t="n"/>
+      <c r="P31" s="24" t="n"/>
+      <c r="Q31" s="25" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="13">
+      <c r="B32" s="15">
         <f>G10</f>
         <v/>
       </c>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="17" t="n"/>
-      <c r="E32" s="17" t="n"/>
-      <c r="F32" s="17" t="n"/>
-      <c r="G32" s="17" t="n"/>
-      <c r="H32" s="17" t="n"/>
-      <c r="I32" s="17" t="n"/>
-      <c r="J32" s="17" t="n"/>
-      <c r="K32" s="17" t="n"/>
-      <c r="L32" s="17" t="n"/>
-      <c r="N32" s="15" t="inlineStr">
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="18" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="18" t="n"/>
+      <c r="J32" s="18" t="n"/>
+      <c r="K32" s="18" t="n"/>
+      <c r="L32" s="18" t="n"/>
+      <c r="N32" s="17" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="O32" s="23" t="n"/>
-      <c r="P32" s="23" t="n"/>
-      <c r="Q32" s="24" t="n"/>
+      <c r="O32" s="24" t="n"/>
+      <c r="P32" s="24" t="n"/>
+      <c r="Q32" s="25" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="C33" s="28" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-      <c r="H33" s="17" t="n"/>
-      <c r="I33" s="17" t="n"/>
-      <c r="J33" s="17" t="n"/>
-      <c r="K33" s="17" t="n"/>
-      <c r="L33" s="17" t="n"/>
-      <c r="N33" s="13">
+      <c r="C33" s="39" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="18" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="18" t="n"/>
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="18" t="n"/>
+      <c r="L33" s="18" t="n"/>
+      <c r="N33" s="15">
         <f>J10</f>
         <v/>
       </c>
-      <c r="O33" s="23" t="n"/>
-      <c r="P33" s="23" t="n"/>
-      <c r="Q33" s="24" t="n"/>
+      <c r="O33" s="24" t="n"/>
+      <c r="P33" s="24" t="n"/>
+      <c r="Q33" s="25" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="13">
+      <c r="B34" s="15">
         <f>H10</f>
         <v/>
       </c>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="17" t="n"/>
-      <c r="E34" s="17" t="n"/>
-      <c r="F34" s="17" t="n"/>
-      <c r="G34" s="17" t="n"/>
-      <c r="H34" s="17" t="n"/>
-      <c r="I34" s="17" t="n"/>
-      <c r="J34" s="17" t="n"/>
-      <c r="K34" s="17" t="n"/>
-      <c r="L34" s="17" t="n"/>
-      <c r="N34" s="17" t="n"/>
-      <c r="O34" s="23" t="n"/>
-      <c r="P34" s="23" t="n"/>
-      <c r="Q34" s="24" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="18" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="18" t="n"/>
+      <c r="L34" s="18" t="n"/>
+      <c r="N34" s="18" t="n"/>
+      <c r="O34" s="24" t="n"/>
+      <c r="P34" s="24" t="n"/>
+      <c r="Q34" s="25" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="C35" s="28" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="17" t="n"/>
-      <c r="H35" s="17" t="n"/>
-      <c r="I35" s="17" t="n"/>
-      <c r="J35" s="17" t="n"/>
-      <c r="K35" s="17" t="n"/>
-      <c r="L35" s="17" t="n"/>
-      <c r="N35" s="17" t="n"/>
-      <c r="O35" s="23" t="n"/>
-      <c r="P35" s="23" t="n"/>
-      <c r="Q35" s="24" t="n"/>
+      <c r="C35" s="39" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="18" t="n"/>
+      <c r="L35" s="18" t="n"/>
+      <c r="N35" s="18" t="n"/>
+      <c r="O35" s="24" t="n"/>
+      <c r="P35" s="24" t="n"/>
+      <c r="Q35" s="25" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="13">
+      <c r="B36" s="15">
         <f>I10</f>
         <v/>
       </c>
-      <c r="C36" s="17" t="n"/>
-      <c r="D36" s="17" t="n"/>
-      <c r="E36" s="17" t="n"/>
-      <c r="F36" s="17" t="n"/>
-      <c r="G36" s="17" t="n"/>
-      <c r="H36" s="17" t="n"/>
-      <c r="I36" s="17" t="n"/>
-      <c r="J36" s="17" t="n"/>
-      <c r="K36" s="17" t="n"/>
-      <c r="L36" s="17" t="n"/>
-      <c r="N36" s="15" t="inlineStr">
+      <c r="C36" s="18" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="18" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="18" t="n"/>
+      <c r="J36" s="18" t="n"/>
+      <c r="K36" s="18" t="n"/>
+      <c r="L36" s="18" t="n"/>
+      <c r="N36" s="17" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="O36" s="23" t="n"/>
-      <c r="P36" s="23" t="n"/>
-      <c r="Q36" s="24" t="n"/>
+      <c r="O36" s="24" t="n"/>
+      <c r="P36" s="24" t="n"/>
+      <c r="Q36" s="25" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="C37" s="28" t="n"/>
-      <c r="D37" s="17" t="n"/>
-      <c r="E37" s="17" t="n"/>
-      <c r="F37" s="17" t="n"/>
-      <c r="G37" s="17" t="n"/>
-      <c r="H37" s="17" t="n"/>
-      <c r="I37" s="17" t="n"/>
-      <c r="J37" s="17" t="n"/>
-      <c r="K37" s="17" t="n"/>
-      <c r="L37" s="17" t="n"/>
-      <c r="N37" s="13">
+      <c r="C37" s="39" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="18" t="n"/>
+      <c r="H37" s="18" t="n"/>
+      <c r="I37" s="18" t="n"/>
+      <c r="J37" s="18" t="n"/>
+      <c r="K37" s="18" t="n"/>
+      <c r="L37" s="18" t="n"/>
+      <c r="N37" s="15">
         <f>K10</f>
         <v/>
       </c>
-      <c r="O37" s="23" t="n"/>
-      <c r="P37" s="23" t="n"/>
-      <c r="Q37" s="24" t="n"/>
+      <c r="O37" s="24" t="n"/>
+      <c r="P37" s="24" t="n"/>
+      <c r="Q37" s="25" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="13">
+      <c r="B38" s="15">
         <f>J10</f>
         <v/>
       </c>
-      <c r="C38" s="17" t="n"/>
-      <c r="D38" s="17" t="n"/>
-      <c r="E38" s="17" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="17" t="n"/>
-      <c r="H38" s="17" t="n"/>
-      <c r="I38" s="17" t="n"/>
-      <c r="J38" s="17" t="n"/>
-      <c r="K38" s="17" t="n"/>
-      <c r="L38" s="17" t="n"/>
-      <c r="N38" s="17" t="n"/>
-      <c r="O38" s="23" t="n"/>
-      <c r="P38" s="23" t="n"/>
-      <c r="Q38" s="24" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="18" t="n"/>
+      <c r="J38" s="18" t="n"/>
+      <c r="K38" s="18" t="n"/>
+      <c r="L38" s="18" t="n"/>
+      <c r="N38" s="18" t="n"/>
+      <c r="O38" s="24" t="n"/>
+      <c r="P38" s="24" t="n"/>
+      <c r="Q38" s="25" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="C39" s="28" t="n"/>
-      <c r="D39" s="17" t="n"/>
-      <c r="E39" s="17" t="n"/>
-      <c r="F39" s="17" t="n"/>
-      <c r="G39" s="17" t="n"/>
-      <c r="H39" s="17" t="n"/>
-      <c r="I39" s="17" t="n"/>
-      <c r="J39" s="17" t="n"/>
-      <c r="K39" s="17" t="n"/>
-      <c r="L39" s="17" t="n"/>
-      <c r="N39" s="17" t="n"/>
-      <c r="O39" s="23" t="n"/>
-      <c r="P39" s="23" t="n"/>
-      <c r="Q39" s="24" t="n"/>
+      <c r="C39" s="39" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="18" t="n"/>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="18" t="n"/>
+      <c r="H39" s="18" t="n"/>
+      <c r="I39" s="18" t="n"/>
+      <c r="J39" s="18" t="n"/>
+      <c r="K39" s="18" t="n"/>
+      <c r="L39" s="18" t="n"/>
+      <c r="N39" s="18" t="n"/>
+      <c r="O39" s="24" t="n"/>
+      <c r="P39" s="24" t="n"/>
+      <c r="Q39" s="25" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="B40" s="13">
+      <c r="B40" s="15">
         <f>K10</f>
         <v/>
       </c>
-      <c r="C40" s="17" t="n"/>
-      <c r="D40" s="17" t="n"/>
-      <c r="E40" s="17" t="n"/>
-      <c r="F40" s="17" t="n"/>
-      <c r="G40" s="17" t="n"/>
-      <c r="H40" s="17" t="n"/>
-      <c r="I40" s="17" t="n"/>
-      <c r="J40" s="17" t="n"/>
-      <c r="K40" s="17" t="n"/>
-      <c r="L40" s="17" t="n"/>
-      <c r="N40" s="29" t="inlineStr">
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="18" t="n"/>
+      <c r="H40" s="18" t="n"/>
+      <c r="I40" s="18" t="n"/>
+      <c r="J40" s="18" t="n"/>
+      <c r="K40" s="18" t="n"/>
+      <c r="L40" s="18" t="n"/>
+      <c r="N40" s="40" t="inlineStr">
         <is>
           <t>Total kilometres</t>
         </is>
       </c>
-      <c r="O40" s="16" t="n"/>
-      <c r="P40" s="16" t="n"/>
-      <c r="Q40" s="26">
+      <c r="O40" s="13" t="n"/>
+      <c r="P40" s="13" t="n"/>
+      <c r="Q40" s="27">
         <f>SUM(Q12:Q39)</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="8" customHeight="1"/>
     <row r="42">
-      <c r="B42" s="30" t="inlineStr">
+      <c r="B42" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C42" s="16" t="n"/>
-      <c r="D42" s="16" t="n"/>
-      <c r="E42" s="16" t="n"/>
-      <c r="G42" s="30" t="inlineStr">
+      <c r="C42" s="13" t="n"/>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
+      <c r="G42" s="41" t="inlineStr">
         <is>
           <t>For approval — client</t>
         </is>
       </c>
-      <c r="H42" s="16" t="n"/>
-      <c r="I42" s="16" t="n"/>
-      <c r="J42" s="16" t="n"/>
-      <c r="K42" s="16" t="n"/>
-      <c r="L42" s="16" t="n"/>
-      <c r="N42" s="30" t="inlineStr">
+      <c r="H42" s="13" t="n"/>
+      <c r="I42" s="13" t="n"/>
+      <c r="J42" s="13" t="n"/>
+      <c r="K42" s="13" t="n"/>
+      <c r="L42" s="13" t="n"/>
+      <c r="N42" s="41" t="inlineStr">
         <is>
           <t>Client signature for approval</t>
         </is>
       </c>
-      <c r="O42" s="16" t="n"/>
-      <c r="P42" s="16" t="n"/>
-      <c r="Q42" s="16" t="n"/>
+      <c r="O42" s="13" t="n"/>
+      <c r="P42" s="13" t="n"/>
+      <c r="Q42" s="13" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="31" t="inlineStr">
+      <c r="B43" s="42" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C43" s="17" t="n"/>
-      <c r="D43" s="17" t="n"/>
-      <c r="E43" s="17" t="n"/>
-      <c r="G43" s="31" t="inlineStr">
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="G43" s="42" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="H43" s="17" t="n"/>
-      <c r="I43" s="17" t="n"/>
-      <c r="J43" s="17" t="n"/>
-      <c r="K43" s="17" t="n"/>
-      <c r="L43" s="17" t="n"/>
-      <c r="N43" s="17" t="n"/>
-      <c r="O43" s="17" t="n"/>
-      <c r="P43" s="17" t="n"/>
-      <c r="Q43" s="17" t="n"/>
+      <c r="H43" s="18" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+      <c r="K43" s="18" t="n"/>
+      <c r="L43" s="18" t="n"/>
+      <c r="N43" s="18" t="n"/>
+      <c r="O43" s="18" t="n"/>
+      <c r="P43" s="18" t="n"/>
+      <c r="Q43" s="18" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="31" t="inlineStr">
+      <c r="B44" s="42" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C44" s="17" t="n"/>
-      <c r="D44" s="17" t="n"/>
-      <c r="E44" s="17" t="n"/>
-      <c r="G44" s="31" t="inlineStr">
+      <c r="C44" s="18" t="n"/>
+      <c r="D44" s="18" t="n"/>
+      <c r="E44" s="18" t="n"/>
+      <c r="G44" s="42" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="H44" s="17" t="n"/>
-      <c r="I44" s="17" t="n"/>
-      <c r="J44" s="17" t="n"/>
-      <c r="K44" s="17" t="n"/>
-      <c r="L44" s="17" t="n"/>
-      <c r="N44" s="17" t="n"/>
-      <c r="O44" s="17" t="n"/>
-      <c r="P44" s="17" t="n"/>
-      <c r="Q44" s="17" t="n"/>
+      <c r="H44" s="18" t="n"/>
+      <c r="I44" s="18" t="n"/>
+      <c r="J44" s="18" t="n"/>
+      <c r="K44" s="18" t="n"/>
+      <c r="L44" s="18" t="n"/>
+      <c r="N44" s="18" t="n"/>
+      <c r="O44" s="18" t="n"/>
+      <c r="P44" s="18" t="n"/>
+      <c r="Q44" s="18" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="31" t="inlineStr">
+      <c r="B45" s="42" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="C45" s="17" t="n"/>
-      <c r="D45" s="17" t="n"/>
-      <c r="E45" s="17" t="n"/>
-      <c r="G45" s="31" t="inlineStr">
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="18" t="n"/>
+      <c r="G45" s="42" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="H45" s="17" t="n"/>
-      <c r="I45" s="17" t="n"/>
-      <c r="J45" s="17" t="n"/>
-      <c r="K45" s="17" t="n"/>
-      <c r="L45" s="17" t="n"/>
-      <c r="N45" s="17" t="n"/>
-      <c r="O45" s="17" t="n"/>
-      <c r="P45" s="17" t="n"/>
-      <c r="Q45" s="17" t="n"/>
+      <c r="H45" s="18" t="n"/>
+      <c r="I45" s="18" t="n"/>
+      <c r="J45" s="18" t="n"/>
+      <c r="K45" s="18" t="n"/>
+      <c r="L45" s="18" t="n"/>
+      <c r="N45" s="18" t="n"/>
+      <c r="O45" s="18" t="n"/>
+      <c r="P45" s="18" t="n"/>
+      <c r="Q45" s="18" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="17" t="n"/>
-      <c r="C46" s="17" t="n"/>
-      <c r="D46" s="17" t="n"/>
-      <c r="E46" s="17" t="n"/>
-      <c r="G46" s="31" t="inlineStr">
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="18" t="n"/>
+      <c r="G46" s="42" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="H46" s="17" t="n"/>
-      <c r="I46" s="17" t="n"/>
-      <c r="J46" s="17" t="n"/>
-      <c r="K46" s="17" t="n"/>
-      <c r="L46" s="17" t="n"/>
-      <c r="N46" s="17" t="n"/>
-      <c r="O46" s="17" t="n"/>
-      <c r="P46" s="17" t="n"/>
-      <c r="Q46" s="17" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="18" t="n"/>
+      <c r="K46" s="18" t="n"/>
+      <c r="L46" s="18" t="n"/>
+      <c r="N46" s="18" t="n"/>
+      <c r="O46" s="18" t="n"/>
+      <c r="P46" s="18" t="n"/>
+      <c r="Q46" s="18" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="17" t="n"/>
-      <c r="C47" s="17" t="n"/>
-      <c r="D47" s="17" t="n"/>
-      <c r="E47" s="17" t="n"/>
-      <c r="N47" s="17" t="n"/>
-      <c r="O47" s="17" t="n"/>
-      <c r="P47" s="17" t="n"/>
-      <c r="Q47" s="17" t="n"/>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="18" t="n"/>
+      <c r="D47" s="18" t="n"/>
+      <c r="E47" s="18" t="n"/>
+      <c r="N47" s="18" t="n"/>
+      <c r="O47" s="18" t="n"/>
+      <c r="P47" s="18" t="n"/>
+      <c r="Q47" s="18" t="n"/>
     </row>
     <row r="48"/>
     <row r="49">
-      <c r="B49" s="32" t="inlineStr">
+      <c r="B49" s="43" t="inlineStr">
         <is>
           <t>Only timesheets signed by the client are processed. One timesheet per week, as PDF or clear photo to admin@q4s.nl.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="47">
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="N37:N39"/>
     <mergeCell ref="N13:N15"/>
@@ -1834,18 +1935,19 @@
     <mergeCell ref="N10:Q10"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="N21:N23"/>
+    <mergeCell ref="B20:D20"/>
     <mergeCell ref="I45:L45"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="C37:L38"/>
     <mergeCell ref="B42:E42"/>
     <mergeCell ref="B8:Q8"/>
+    <mergeCell ref="B9:L9"/>
     <mergeCell ref="G44:H44"/>
     <mergeCell ref="C31:L32"/>
     <mergeCell ref="L10:L11"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="C33:L34"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="B20:L20"/>
     <mergeCell ref="N40:P40"/>
     <mergeCell ref="N17:N19"/>
     <mergeCell ref="G45:H45"/>

</xml_diff>

<commit_message>
Q4S-Timesheet: alleen weeknummer invullen; Van/Tot en alle datums (rooster, omschrijving per dag, kilometers) rekenen automatisch (ISO-week, huidig jaar met jaarwissel-correctie)
</commit_message>
<xml_diff>
--- a/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
+++ b/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -268,12 +268,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -324,6 +318,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -819,7 +816,10 @@
           <t>From</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="n"/>
+      <c r="Q2" s="6">
+        <f>IF(O4="","",DATE(YEAR(TODAY())+IF(AND(MONTH(TODAY())=12,O4&lt;10),1,IF(AND(MONTH(TODAY())=1,O4&gt;40),-1,0)),1,4)-WEEKDAY(DATE(YEAR(TODAY())+IF(AND(MONTH(TODAY())=12,O4&lt;10),1,IF(AND(MONTH(TODAY())=1,O4&gt;40),-1,0)),1,4),3)+7*(O4-1))</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="C3" s="3" t="inlineStr">
@@ -859,16 +859,13 @@
           <t>Week no.</t>
         </is>
       </c>
-      <c r="O4" s="7">
-        <f>IF(Q2="","",_xlfn.ISOWEEKNUM(Q2))</f>
-        <v/>
-      </c>
+      <c r="O4" s="5" t="n"/>
       <c r="P4" s="4" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="Q4" s="8">
+      <c r="Q4" s="6">
         <f>IF(Q2="","",Q2+6)</f>
         <v/>
       </c>
@@ -884,7 +881,7 @@
           <t>E-mail</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>admin@q4s.nl</t>
         </is>
@@ -911,996 +908,996 @@
     </row>
     <row r="7" ht="6" customHeight="1"/>
     <row r="8" ht="20" customHeight="1">
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Send the signed timesheet every week to admin@q4s.nl — no later than Tuesday 12:00</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
-      <c r="O8" s="11" t="n"/>
-      <c r="P8" s="11" t="n"/>
-      <c r="Q8" s="11" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
+      <c r="O8" s="9" t="n"/>
+      <c r="P8" s="9" t="n"/>
+      <c r="Q8" s="9" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>NORMAL HOURS — regular hours per day. Hours above the regular schedule go in the orange OVERTIME block below.</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
-      <c r="K9" s="13" t="n"/>
-      <c r="L9" s="13" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Client / Proj. no.</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Hour code</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="13">
         <f>IF(Q2="","",Q2+0)</f>
         <v/>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="13">
         <f>IF(Q2="","",Q2+1)</f>
         <v/>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="13">
         <f>IF(Q2="","",Q2+2)</f>
         <v/>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="13">
         <f>IF(Q2="","",Q2+3)</f>
         <v/>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="13">
         <f>IF(Q2="","",Q2+4)</f>
         <v/>
       </c>
-      <c r="J10" s="15">
+      <c r="J10" s="13">
         <f>IF(Q2="","",Q2+5)</f>
         <v/>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="13">
         <f>IF(Q2="","",Q2+6)</f>
         <v/>
       </c>
-      <c r="L10" s="16" t="inlineStr">
+      <c r="L10" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="N10" s="17" t="inlineStr">
+      <c r="N10" s="15" t="inlineStr">
         <is>
           <t>Kilometres</t>
         </is>
       </c>
-      <c r="O10" s="13" t="n"/>
-      <c r="P10" s="13" t="n"/>
-      <c r="Q10" s="13" t="n"/>
+      <c r="O10" s="11" t="n"/>
+      <c r="P10" s="11" t="n"/>
+      <c r="Q10" s="11" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="18" t="n"/>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="15" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="K11" s="17" t="inlineStr">
+      <c r="K11" s="15" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="L11" s="18" t="n"/>
-      <c r="N11" s="19" t="inlineStr"/>
-      <c r="O11" s="19" t="inlineStr">
+      <c r="L11" s="16" t="n"/>
+      <c r="N11" s="17" t="inlineStr"/>
+      <c r="O11" s="17" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="P11" s="19" t="inlineStr">
+      <c r="P11" s="17" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="Q11" s="19" t="inlineStr">
+      <c r="Q11" s="17" t="inlineStr">
         <is>
           <t>Km</t>
         </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="22" t="n"/>
-      <c r="K12" s="22" t="n"/>
-      <c r="L12" s="23">
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+      <c r="H12" s="19" t="n"/>
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="20" t="n"/>
+      <c r="K12" s="20" t="n"/>
+      <c r="L12" s="21">
         <f>IF(SUM(E12:K12)=0,"",SUM(E12:K12))</f>
         <v/>
       </c>
-      <c r="N12" s="17" t="inlineStr">
+      <c r="N12" s="15" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="O12" s="24" t="n"/>
-      <c r="P12" s="24" t="n"/>
-      <c r="Q12" s="25" t="n"/>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="22" t="n"/>
+      <c r="Q12" s="23" t="n"/>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="21" t="n"/>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="21" t="n"/>
-      <c r="J13" s="22" t="n"/>
-      <c r="K13" s="22" t="n"/>
-      <c r="L13" s="23">
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="20" t="n"/>
+      <c r="K13" s="20" t="n"/>
+      <c r="L13" s="21">
         <f>IF(SUM(E13:K13)=0,"",SUM(E13:K13))</f>
         <v/>
       </c>
-      <c r="N13" s="15">
+      <c r="N13" s="13">
         <f>E10</f>
         <v/>
       </c>
-      <c r="O13" s="24" t="n"/>
-      <c r="P13" s="24" t="n"/>
-      <c r="Q13" s="25" t="n"/>
+      <c r="O13" s="22" t="n"/>
+      <c r="P13" s="22" t="n"/>
+      <c r="Q13" s="23" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="21" t="n"/>
-      <c r="H14" s="21" t="n"/>
-      <c r="I14" s="21" t="n"/>
-      <c r="J14" s="22" t="n"/>
-      <c r="K14" s="22" t="n"/>
-      <c r="L14" s="23">
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="20" t="n"/>
+      <c r="K14" s="20" t="n"/>
+      <c r="L14" s="21">
         <f>IF(SUM(E14:K14)=0,"",SUM(E14:K14))</f>
         <v/>
       </c>
-      <c r="N14" s="18" t="n"/>
-      <c r="O14" s="24" t="n"/>
-      <c r="P14" s="24" t="n"/>
-      <c r="Q14" s="25" t="n"/>
+      <c r="N14" s="16" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="22" t="n"/>
+      <c r="Q14" s="23" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="21" t="n"/>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="21" t="n"/>
-      <c r="J15" s="22" t="n"/>
-      <c r="K15" s="22" t="n"/>
-      <c r="L15" s="23">
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="20" t="n"/>
+      <c r="K15" s="20" t="n"/>
+      <c r="L15" s="21">
         <f>IF(SUM(E15:K15)=0,"",SUM(E15:K15))</f>
         <v/>
       </c>
-      <c r="N15" s="18" t="n"/>
-      <c r="O15" s="24" t="n"/>
-      <c r="P15" s="24" t="n"/>
-      <c r="Q15" s="25" t="n"/>
+      <c r="N15" s="16" t="n"/>
+      <c r="O15" s="22" t="n"/>
+      <c r="P15" s="22" t="n"/>
+      <c r="Q15" s="23" t="n"/>
     </row>
     <row r="16" ht="17" customHeight="1">
-      <c r="B16" s="20" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="21" t="n"/>
-      <c r="G16" s="21" t="n"/>
-      <c r="H16" s="21" t="n"/>
-      <c r="I16" s="21" t="n"/>
-      <c r="J16" s="22" t="n"/>
-      <c r="K16" s="22" t="n"/>
-      <c r="L16" s="23">
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="20" t="n"/>
+      <c r="K16" s="20" t="n"/>
+      <c r="L16" s="21">
         <f>IF(SUM(E16:K16)=0,"",SUM(E16:K16))</f>
         <v/>
       </c>
-      <c r="N16" s="17" t="inlineStr">
+      <c r="N16" s="15" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="O16" s="24" t="n"/>
-      <c r="P16" s="24" t="n"/>
-      <c r="Q16" s="25" t="n"/>
+      <c r="O16" s="22" t="n"/>
+      <c r="P16" s="22" t="n"/>
+      <c r="Q16" s="23" t="n"/>
     </row>
     <row r="17" ht="17" customHeight="1">
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="21" t="n"/>
-      <c r="G17" s="21" t="n"/>
-      <c r="H17" s="21" t="n"/>
-      <c r="I17" s="21" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="22" t="n"/>
-      <c r="L17" s="23">
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="20" t="n"/>
+      <c r="K17" s="20" t="n"/>
+      <c r="L17" s="21">
         <f>IF(SUM(E17:K17)=0,"",SUM(E17:K17))</f>
         <v/>
       </c>
-      <c r="N17" s="15">
+      <c r="N17" s="13">
         <f>F10</f>
         <v/>
       </c>
-      <c r="O17" s="24" t="n"/>
-      <c r="P17" s="24" t="n"/>
-      <c r="Q17" s="25" t="n"/>
+      <c r="O17" s="22" t="n"/>
+      <c r="P17" s="22" t="n"/>
+      <c r="Q17" s="23" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="26" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Total normal hours</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="7">
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="25">
         <f>SUM(E12:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="25">
         <f>SUM(F12:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="25">
         <f>SUM(G12:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="25">
         <f>SUM(H12:H17)</f>
         <v/>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="25">
         <f>SUM(I12:I17)</f>
         <v/>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="25">
         <f>SUM(J12:J17)</f>
         <v/>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="25">
         <f>SUM(K12:K17)</f>
         <v/>
       </c>
-      <c r="L18" s="27">
+      <c r="L18" s="26">
         <f>SUM(E18:K18)</f>
         <v/>
       </c>
-      <c r="N18" s="18" t="n"/>
-      <c r="O18" s="24" t="n"/>
-      <c r="P18" s="24" t="n"/>
-      <c r="Q18" s="25" t="n"/>
+      <c r="N18" s="16" t="n"/>
+      <c r="O18" s="22" t="n"/>
+      <c r="P18" s="22" t="n"/>
+      <c r="Q18" s="23" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="24" t="n"/>
-      <c r="P19" s="24" t="n"/>
-      <c r="Q19" s="25" t="n"/>
+      <c r="N19" s="16" t="n"/>
+      <c r="O19" s="22" t="n"/>
+      <c r="P19" s="22" t="n"/>
+      <c r="Q19" s="23" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>OVERTIME (extra hrs)</t>
         </is>
       </c>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="30" t="inlineStr">
+      <c r="C20" s="28" t="n"/>
+      <c r="D20" s="28" t="n"/>
+      <c r="E20" s="29" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="F20" s="30" t="inlineStr">
+      <c r="F20" s="29" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="G20" s="30" t="inlineStr">
+      <c r="G20" s="29" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="H20" s="30" t="inlineStr">
+      <c r="H20" s="29" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="I20" s="30" t="inlineStr">
+      <c r="I20" s="29" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="J20" s="30" t="inlineStr">
+      <c r="J20" s="29" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="K20" s="30" t="inlineStr">
+      <c r="K20" s="29" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="L20" s="31" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="N20" s="17" t="inlineStr">
+      <c r="N20" s="15" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="O20" s="24" t="n"/>
-      <c r="P20" s="24" t="n"/>
-      <c r="Q20" s="25" t="n"/>
+      <c r="O20" s="22" t="n"/>
+      <c r="P20" s="22" t="n"/>
+      <c r="Q20" s="23" t="n"/>
     </row>
     <row r="21" ht="17" customHeight="1">
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="33" t="n"/>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
-      <c r="G21" s="33" t="n"/>
-      <c r="H21" s="33" t="n"/>
-      <c r="I21" s="33" t="n"/>
-      <c r="J21" s="33" t="n"/>
-      <c r="K21" s="33" t="n"/>
-      <c r="L21" s="34">
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
+      <c r="K21" s="32" t="n"/>
+      <c r="L21" s="33">
         <f>IF(SUM(E21:K21)=0,"",SUM(E21:K21))</f>
         <v/>
       </c>
-      <c r="N21" s="15">
+      <c r="N21" s="13">
         <f>G10</f>
         <v/>
       </c>
-      <c r="O21" s="24" t="n"/>
-      <c r="P21" s="24" t="n"/>
-      <c r="Q21" s="25" t="n"/>
+      <c r="O21" s="22" t="n"/>
+      <c r="P21" s="22" t="n"/>
+      <c r="Q21" s="23" t="n"/>
     </row>
     <row r="22" ht="17" customHeight="1">
-      <c r="B22" s="32" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="33" t="n"/>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="33" t="n"/>
-      <c r="G22" s="33" t="n"/>
-      <c r="H22" s="33" t="n"/>
-      <c r="I22" s="33" t="n"/>
-      <c r="J22" s="33" t="n"/>
-      <c r="K22" s="33" t="n"/>
-      <c r="L22" s="34">
+      <c r="B22" s="31" t="n"/>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="32" t="n"/>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="32" t="n"/>
+      <c r="I22" s="32" t="n"/>
+      <c r="J22" s="32" t="n"/>
+      <c r="K22" s="32" t="n"/>
+      <c r="L22" s="33">
         <f>IF(SUM(E22:K22)=0,"",SUM(E22:K22))</f>
         <v/>
       </c>
-      <c r="N22" s="18" t="n"/>
-      <c r="O22" s="24" t="n"/>
-      <c r="P22" s="24" t="n"/>
-      <c r="Q22" s="25" t="n"/>
+      <c r="N22" s="16" t="n"/>
+      <c r="O22" s="22" t="n"/>
+      <c r="P22" s="22" t="n"/>
+      <c r="Q22" s="23" t="n"/>
     </row>
     <row r="23" ht="17" customHeight="1">
-      <c r="B23" s="32" t="n"/>
-      <c r="C23" s="33" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
-      <c r="G23" s="33" t="n"/>
-      <c r="H23" s="33" t="n"/>
-      <c r="I23" s="33" t="n"/>
-      <c r="J23" s="33" t="n"/>
-      <c r="K23" s="33" t="n"/>
-      <c r="L23" s="34">
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="32" t="n"/>
+      <c r="J23" s="32" t="n"/>
+      <c r="K23" s="32" t="n"/>
+      <c r="L23" s="33">
         <f>IF(SUM(E23:K23)=0,"",SUM(E23:K23))</f>
         <v/>
       </c>
-      <c r="N23" s="18" t="n"/>
-      <c r="O23" s="24" t="n"/>
-      <c r="P23" s="24" t="n"/>
-      <c r="Q23" s="25" t="n"/>
+      <c r="N23" s="16" t="n"/>
+      <c r="O23" s="22" t="n"/>
+      <c r="P23" s="22" t="n"/>
+      <c r="Q23" s="23" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>Total overtime</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="36">
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="35">
         <f>SUM(E21:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="36">
+      <c r="F24" s="35">
         <f>SUM(F21:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="36">
+      <c r="G24" s="35">
         <f>SUM(G21:G23)</f>
         <v/>
       </c>
-      <c r="H24" s="36">
+      <c r="H24" s="35">
         <f>SUM(H21:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="36">
+      <c r="I24" s="35">
         <f>SUM(I21:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="36">
+      <c r="J24" s="35">
         <f>SUM(J21:J23)</f>
         <v/>
       </c>
-      <c r="K24" s="36">
+      <c r="K24" s="35">
         <f>SUM(K21:K23)</f>
         <v/>
       </c>
-      <c r="L24" s="37">
+      <c r="L24" s="36">
         <f>SUM(E24:K24)</f>
         <v/>
       </c>
-      <c r="N24" s="17" t="inlineStr">
+      <c r="N24" s="15" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="O24" s="24" t="n"/>
-      <c r="P24" s="24" t="n"/>
-      <c r="Q24" s="25" t="n"/>
+      <c r="O24" s="22" t="n"/>
+      <c r="P24" s="22" t="n"/>
+      <c r="Q24" s="23" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="N25" s="15">
+      <c r="N25" s="13">
         <f>H10</f>
         <v/>
       </c>
-      <c r="O25" s="24" t="n"/>
-      <c r="P25" s="24" t="n"/>
-      <c r="Q25" s="25" t="n"/>
+      <c r="O25" s="22" t="n"/>
+      <c r="P25" s="22" t="n"/>
+      <c r="Q25" s="23" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C26" s="38" t="inlineStr">
+      <c r="C26" s="37" t="inlineStr">
         <is>
           <t>Description of work</t>
         </is>
       </c>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
-      <c r="H26" s="11" t="n"/>
-      <c r="I26" s="11" t="n"/>
-      <c r="J26" s="11" t="n"/>
-      <c r="K26" s="11" t="n"/>
-      <c r="L26" s="11" t="n"/>
-      <c r="N26" s="18" t="n"/>
-      <c r="O26" s="24" t="n"/>
-      <c r="P26" s="24" t="n"/>
-      <c r="Q26" s="25" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="N26" s="16" t="n"/>
+      <c r="O26" s="22" t="n"/>
+      <c r="P26" s="22" t="n"/>
+      <c r="Q26" s="23" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="C27" s="39" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="N27" s="18" t="n"/>
-      <c r="O27" s="24" t="n"/>
-      <c r="P27" s="24" t="n"/>
-      <c r="Q27" s="25" t="n"/>
+      <c r="C27" s="38" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="16" t="n"/>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="16" t="n"/>
+      <c r="L27" s="16" t="n"/>
+      <c r="N27" s="16" t="n"/>
+      <c r="O27" s="22" t="n"/>
+      <c r="P27" s="22" t="n"/>
+      <c r="Q27" s="23" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="15">
+      <c r="B28" s="13">
         <f>E10</f>
         <v/>
       </c>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="18" t="n"/>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="18" t="n"/>
-      <c r="L28" s="18" t="n"/>
-      <c r="N28" s="17" t="inlineStr">
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="16" t="n"/>
+      <c r="K28" s="16" t="n"/>
+      <c r="L28" s="16" t="n"/>
+      <c r="N28" s="15" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="O28" s="24" t="n"/>
-      <c r="P28" s="24" t="n"/>
-      <c r="Q28" s="25" t="n"/>
+      <c r="O28" s="22" t="n"/>
+      <c r="P28" s="22" t="n"/>
+      <c r="Q28" s="23" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Tu</t>
         </is>
       </c>
-      <c r="C29" s="39" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="18" t="n"/>
-      <c r="I29" s="18" t="n"/>
-      <c r="J29" s="18" t="n"/>
-      <c r="K29" s="18" t="n"/>
-      <c r="L29" s="18" t="n"/>
-      <c r="N29" s="15">
+      <c r="C29" s="38" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="16" t="n"/>
+      <c r="H29" s="16" t="n"/>
+      <c r="I29" s="16" t="n"/>
+      <c r="J29" s="16" t="n"/>
+      <c r="K29" s="16" t="n"/>
+      <c r="L29" s="16" t="n"/>
+      <c r="N29" s="13">
         <f>I10</f>
         <v/>
       </c>
-      <c r="O29" s="24" t="n"/>
-      <c r="P29" s="24" t="n"/>
-      <c r="Q29" s="25" t="n"/>
+      <c r="O29" s="22" t="n"/>
+      <c r="P29" s="22" t="n"/>
+      <c r="Q29" s="23" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="15">
+      <c r="B30" s="13">
         <f>F10</f>
         <v/>
       </c>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="18" t="n"/>
-      <c r="K30" s="18" t="n"/>
-      <c r="L30" s="18" t="n"/>
-      <c r="N30" s="18" t="n"/>
-      <c r="O30" s="24" t="n"/>
-      <c r="P30" s="24" t="n"/>
-      <c r="Q30" s="25" t="n"/>
+      <c r="C30" s="16" t="n"/>
+      <c r="D30" s="16" t="n"/>
+      <c r="E30" s="16" t="n"/>
+      <c r="F30" s="16" t="n"/>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="16" t="n"/>
+      <c r="I30" s="16" t="n"/>
+      <c r="J30" s="16" t="n"/>
+      <c r="K30" s="16" t="n"/>
+      <c r="L30" s="16" t="n"/>
+      <c r="N30" s="16" t="n"/>
+      <c r="O30" s="22" t="n"/>
+      <c r="P30" s="22" t="n"/>
+      <c r="Q30" s="23" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>We</t>
         </is>
       </c>
-      <c r="C31" s="39" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="18" t="n"/>
-      <c r="L31" s="18" t="n"/>
-      <c r="N31" s="18" t="n"/>
-      <c r="O31" s="24" t="n"/>
-      <c r="P31" s="24" t="n"/>
-      <c r="Q31" s="25" t="n"/>
+      <c r="C31" s="38" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="16" t="n"/>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="n"/>
+      <c r="J31" s="16" t="n"/>
+      <c r="K31" s="16" t="n"/>
+      <c r="L31" s="16" t="n"/>
+      <c r="N31" s="16" t="n"/>
+      <c r="O31" s="22" t="n"/>
+      <c r="P31" s="22" t="n"/>
+      <c r="Q31" s="23" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="15">
+      <c r="B32" s="13">
         <f>G10</f>
         <v/>
       </c>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="18" t="n"/>
-      <c r="L32" s="18" t="n"/>
-      <c r="N32" s="17" t="inlineStr">
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
+      <c r="J32" s="16" t="n"/>
+      <c r="K32" s="16" t="n"/>
+      <c r="L32" s="16" t="n"/>
+      <c r="N32" s="15" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="O32" s="24" t="n"/>
-      <c r="P32" s="24" t="n"/>
-      <c r="Q32" s="25" t="n"/>
+      <c r="O32" s="22" t="n"/>
+      <c r="P32" s="22" t="n"/>
+      <c r="Q32" s="23" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="C33" s="39" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
-      <c r="J33" s="18" t="n"/>
-      <c r="K33" s="18" t="n"/>
-      <c r="L33" s="18" t="n"/>
-      <c r="N33" s="15">
+      <c r="C33" s="38" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
+      <c r="H33" s="16" t="n"/>
+      <c r="I33" s="16" t="n"/>
+      <c r="J33" s="16" t="n"/>
+      <c r="K33" s="16" t="n"/>
+      <c r="L33" s="16" t="n"/>
+      <c r="N33" s="13">
         <f>J10</f>
         <v/>
       </c>
-      <c r="O33" s="24" t="n"/>
-      <c r="P33" s="24" t="n"/>
-      <c r="Q33" s="25" t="n"/>
+      <c r="O33" s="22" t="n"/>
+      <c r="P33" s="22" t="n"/>
+      <c r="Q33" s="23" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="15">
+      <c r="B34" s="13">
         <f>H10</f>
         <v/>
       </c>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="18" t="n"/>
-      <c r="I34" s="18" t="n"/>
-      <c r="J34" s="18" t="n"/>
-      <c r="K34" s="18" t="n"/>
-      <c r="L34" s="18" t="n"/>
-      <c r="N34" s="18" t="n"/>
-      <c r="O34" s="24" t="n"/>
-      <c r="P34" s="24" t="n"/>
-      <c r="Q34" s="25" t="n"/>
+      <c r="C34" s="16" t="n"/>
+      <c r="D34" s="16" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="16" t="n"/>
+      <c r="H34" s="16" t="n"/>
+      <c r="I34" s="16" t="n"/>
+      <c r="J34" s="16" t="n"/>
+      <c r="K34" s="16" t="n"/>
+      <c r="L34" s="16" t="n"/>
+      <c r="N34" s="16" t="n"/>
+      <c r="O34" s="22" t="n"/>
+      <c r="P34" s="22" t="n"/>
+      <c r="Q34" s="23" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="C35" s="39" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="18" t="n"/>
-      <c r="I35" s="18" t="n"/>
-      <c r="J35" s="18" t="n"/>
-      <c r="K35" s="18" t="n"/>
-      <c r="L35" s="18" t="n"/>
-      <c r="N35" s="18" t="n"/>
-      <c r="O35" s="24" t="n"/>
-      <c r="P35" s="24" t="n"/>
-      <c r="Q35" s="25" t="n"/>
+      <c r="C35" s="38" t="n"/>
+      <c r="D35" s="16" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="16" t="n"/>
+      <c r="G35" s="16" t="n"/>
+      <c r="H35" s="16" t="n"/>
+      <c r="I35" s="16" t="n"/>
+      <c r="J35" s="16" t="n"/>
+      <c r="K35" s="16" t="n"/>
+      <c r="L35" s="16" t="n"/>
+      <c r="N35" s="16" t="n"/>
+      <c r="O35" s="22" t="n"/>
+      <c r="P35" s="22" t="n"/>
+      <c r="Q35" s="23" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="15">
+      <c r="B36" s="13">
         <f>I10</f>
         <v/>
       </c>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
-      <c r="I36" s="18" t="n"/>
-      <c r="J36" s="18" t="n"/>
-      <c r="K36" s="18" t="n"/>
-      <c r="L36" s="18" t="n"/>
-      <c r="N36" s="17" t="inlineStr">
+      <c r="C36" s="16" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="16" t="n"/>
+      <c r="H36" s="16" t="n"/>
+      <c r="I36" s="16" t="n"/>
+      <c r="J36" s="16" t="n"/>
+      <c r="K36" s="16" t="n"/>
+      <c r="L36" s="16" t="n"/>
+      <c r="N36" s="15" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="O36" s="24" t="n"/>
-      <c r="P36" s="24" t="n"/>
-      <c r="Q36" s="25" t="n"/>
+      <c r="O36" s="22" t="n"/>
+      <c r="P36" s="22" t="n"/>
+      <c r="Q36" s="23" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="C37" s="39" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="18" t="n"/>
-      <c r="L37" s="18" t="n"/>
-      <c r="N37" s="15">
+      <c r="C37" s="38" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="16" t="n"/>
+      <c r="H37" s="16" t="n"/>
+      <c r="I37" s="16" t="n"/>
+      <c r="J37" s="16" t="n"/>
+      <c r="K37" s="16" t="n"/>
+      <c r="L37" s="16" t="n"/>
+      <c r="N37" s="13">
         <f>K10</f>
         <v/>
       </c>
-      <c r="O37" s="24" t="n"/>
-      <c r="P37" s="24" t="n"/>
-      <c r="Q37" s="25" t="n"/>
+      <c r="O37" s="22" t="n"/>
+      <c r="P37" s="22" t="n"/>
+      <c r="Q37" s="23" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="15">
+      <c r="B38" s="13">
         <f>J10</f>
         <v/>
       </c>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="18" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="18" t="n"/>
-      <c r="L38" s="18" t="n"/>
-      <c r="N38" s="18" t="n"/>
-      <c r="O38" s="24" t="n"/>
-      <c r="P38" s="24" t="n"/>
-      <c r="Q38" s="25" t="n"/>
+      <c r="C38" s="16" t="n"/>
+      <c r="D38" s="16" t="n"/>
+      <c r="E38" s="16" t="n"/>
+      <c r="F38" s="16" t="n"/>
+      <c r="G38" s="16" t="n"/>
+      <c r="H38" s="16" t="n"/>
+      <c r="I38" s="16" t="n"/>
+      <c r="J38" s="16" t="n"/>
+      <c r="K38" s="16" t="n"/>
+      <c r="L38" s="16" t="n"/>
+      <c r="N38" s="16" t="n"/>
+      <c r="O38" s="22" t="n"/>
+      <c r="P38" s="22" t="n"/>
+      <c r="Q38" s="23" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
       </c>
-      <c r="C39" s="39" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
-      <c r="H39" s="18" t="n"/>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="18" t="n"/>
-      <c r="L39" s="18" t="n"/>
-      <c r="N39" s="18" t="n"/>
-      <c r="O39" s="24" t="n"/>
-      <c r="P39" s="24" t="n"/>
-      <c r="Q39" s="25" t="n"/>
+      <c r="C39" s="38" t="n"/>
+      <c r="D39" s="16" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="16" t="n"/>
+      <c r="G39" s="16" t="n"/>
+      <c r="H39" s="16" t="n"/>
+      <c r="I39" s="16" t="n"/>
+      <c r="J39" s="16" t="n"/>
+      <c r="K39" s="16" t="n"/>
+      <c r="L39" s="16" t="n"/>
+      <c r="N39" s="16" t="n"/>
+      <c r="O39" s="22" t="n"/>
+      <c r="P39" s="22" t="n"/>
+      <c r="Q39" s="23" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="B40" s="15">
+      <c r="B40" s="13">
         <f>K10</f>
         <v/>
       </c>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-      <c r="G40" s="18" t="n"/>
-      <c r="H40" s="18" t="n"/>
-      <c r="I40" s="18" t="n"/>
-      <c r="J40" s="18" t="n"/>
-      <c r="K40" s="18" t="n"/>
-      <c r="L40" s="18" t="n"/>
-      <c r="N40" s="40" t="inlineStr">
+      <c r="C40" s="16" t="n"/>
+      <c r="D40" s="16" t="n"/>
+      <c r="E40" s="16" t="n"/>
+      <c r="F40" s="16" t="n"/>
+      <c r="G40" s="16" t="n"/>
+      <c r="H40" s="16" t="n"/>
+      <c r="I40" s="16" t="n"/>
+      <c r="J40" s="16" t="n"/>
+      <c r="K40" s="16" t="n"/>
+      <c r="L40" s="16" t="n"/>
+      <c r="N40" s="39" t="inlineStr">
         <is>
           <t>Total kilometres</t>
         </is>
       </c>
-      <c r="O40" s="13" t="n"/>
-      <c r="P40" s="13" t="n"/>
-      <c r="Q40" s="27">
+      <c r="O40" s="11" t="n"/>
+      <c r="P40" s="11" t="n"/>
+      <c r="Q40" s="26">
         <f>SUM(Q12:Q39)</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="8" customHeight="1"/>
     <row r="42">
-      <c r="B42" s="41" t="inlineStr">
+      <c r="B42" s="40" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C42" s="13" t="n"/>
-      <c r="D42" s="13" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="G42" s="41" t="inlineStr">
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="G42" s="40" t="inlineStr">
         <is>
           <t>For approval — client</t>
         </is>
       </c>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="13" t="n"/>
-      <c r="J42" s="13" t="n"/>
-      <c r="K42" s="13" t="n"/>
-      <c r="L42" s="13" t="n"/>
-      <c r="N42" s="41" t="inlineStr">
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="11" t="n"/>
+      <c r="J42" s="11" t="n"/>
+      <c r="K42" s="11" t="n"/>
+      <c r="L42" s="11" t="n"/>
+      <c r="N42" s="40" t="inlineStr">
         <is>
           <t>Client signature for approval</t>
         </is>
       </c>
-      <c r="O42" s="13" t="n"/>
-      <c r="P42" s="13" t="n"/>
-      <c r="Q42" s="13" t="n"/>
+      <c r="O42" s="11" t="n"/>
+      <c r="P42" s="11" t="n"/>
+      <c r="Q42" s="11" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="42" t="inlineStr">
+      <c r="B43" s="41" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="G43" s="42" t="inlineStr">
+      <c r="C43" s="16" t="n"/>
+      <c r="D43" s="16" t="n"/>
+      <c r="E43" s="16" t="n"/>
+      <c r="G43" s="41" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="H43" s="18" t="n"/>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18" t="n"/>
-      <c r="K43" s="18" t="n"/>
-      <c r="L43" s="18" t="n"/>
-      <c r="N43" s="18" t="n"/>
-      <c r="O43" s="18" t="n"/>
-      <c r="P43" s="18" t="n"/>
-      <c r="Q43" s="18" t="n"/>
+      <c r="H43" s="16" t="n"/>
+      <c r="I43" s="16" t="n"/>
+      <c r="J43" s="16" t="n"/>
+      <c r="K43" s="16" t="n"/>
+      <c r="L43" s="16" t="n"/>
+      <c r="N43" s="16" t="n"/>
+      <c r="O43" s="16" t="n"/>
+      <c r="P43" s="16" t="n"/>
+      <c r="Q43" s="16" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="42" t="inlineStr">
+      <c r="B44" s="41" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="G44" s="42" t="inlineStr">
+      <c r="C44" s="16" t="n"/>
+      <c r="D44" s="16" t="n"/>
+      <c r="E44" s="16" t="n"/>
+      <c r="G44" s="41" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="H44" s="18" t="n"/>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18" t="n"/>
-      <c r="K44" s="18" t="n"/>
-      <c r="L44" s="18" t="n"/>
-      <c r="N44" s="18" t="n"/>
-      <c r="O44" s="18" t="n"/>
-      <c r="P44" s="18" t="n"/>
-      <c r="Q44" s="18" t="n"/>
+      <c r="H44" s="16" t="n"/>
+      <c r="I44" s="16" t="n"/>
+      <c r="J44" s="16" t="n"/>
+      <c r="K44" s="16" t="n"/>
+      <c r="L44" s="16" t="n"/>
+      <c r="N44" s="16" t="n"/>
+      <c r="O44" s="16" t="n"/>
+      <c r="P44" s="16" t="n"/>
+      <c r="Q44" s="16" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="42" t="inlineStr">
+      <c r="B45" s="41" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="C45" s="18" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="18" t="n"/>
-      <c r="G45" s="42" t="inlineStr">
+      <c r="C45" s="16" t="n"/>
+      <c r="D45" s="16" t="n"/>
+      <c r="E45" s="16" t="n"/>
+      <c r="G45" s="41" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="H45" s="18" t="n"/>
-      <c r="I45" s="18" t="n"/>
-      <c r="J45" s="18" t="n"/>
-      <c r="K45" s="18" t="n"/>
-      <c r="L45" s="18" t="n"/>
-      <c r="N45" s="18" t="n"/>
-      <c r="O45" s="18" t="n"/>
-      <c r="P45" s="18" t="n"/>
-      <c r="Q45" s="18" t="n"/>
+      <c r="H45" s="16" t="n"/>
+      <c r="I45" s="16" t="n"/>
+      <c r="J45" s="16" t="n"/>
+      <c r="K45" s="16" t="n"/>
+      <c r="L45" s="16" t="n"/>
+      <c r="N45" s="16" t="n"/>
+      <c r="O45" s="16" t="n"/>
+      <c r="P45" s="16" t="n"/>
+      <c r="Q45" s="16" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="18" t="n"/>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="18" t="n"/>
-      <c r="G46" s="42" t="inlineStr">
+      <c r="B46" s="16" t="n"/>
+      <c r="C46" s="16" t="n"/>
+      <c r="D46" s="16" t="n"/>
+      <c r="E46" s="16" t="n"/>
+      <c r="G46" s="41" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="H46" s="18" t="n"/>
-      <c r="I46" s="18" t="n"/>
-      <c r="J46" s="18" t="n"/>
-      <c r="K46" s="18" t="n"/>
-      <c r="L46" s="18" t="n"/>
-      <c r="N46" s="18" t="n"/>
-      <c r="O46" s="18" t="n"/>
-      <c r="P46" s="18" t="n"/>
-      <c r="Q46" s="18" t="n"/>
+      <c r="H46" s="16" t="n"/>
+      <c r="I46" s="16" t="n"/>
+      <c r="J46" s="16" t="n"/>
+      <c r="K46" s="16" t="n"/>
+      <c r="L46" s="16" t="n"/>
+      <c r="N46" s="16" t="n"/>
+      <c r="O46" s="16" t="n"/>
+      <c r="P46" s="16" t="n"/>
+      <c r="Q46" s="16" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="18" t="n"/>
-      <c r="C47" s="18" t="n"/>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="18" t="n"/>
-      <c r="N47" s="18" t="n"/>
-      <c r="O47" s="18" t="n"/>
-      <c r="P47" s="18" t="n"/>
-      <c r="Q47" s="18" t="n"/>
+      <c r="B47" s="16" t="n"/>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="16" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="N47" s="16" t="n"/>
+      <c r="O47" s="16" t="n"/>
+      <c r="P47" s="16" t="n"/>
+      <c r="Q47" s="16" t="n"/>
     </row>
     <row r="48"/>
     <row r="49">
-      <c r="B49" s="43" t="inlineStr">
+      <c r="B49" s="42" t="inlineStr">
         <is>
           <t>Only timesheets signed by the client are processed. One timesheet per week, as PDF or clear photo to admin@q4s.nl.</t>
         </is>
@@ -1957,8 +1954,9 @@
     <mergeCell ref="C27:L28"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="Q2" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="From" prompt="Enter the date of Monday — dates, week number and 'To' follow automatically." type="date" operator="greaterThan">
-      <formula1>DATE(2020,1,1)</formula1>
+    <dataValidation sqref="O4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Week no." error="Enter the week number (1-53) — From, To and all dates follow automatically." promptTitle="Week no." prompt="Enter the week number (1-53) — From, To and all dates follow automatically." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>53</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
Q4S-Timesheet: breder (alle kolommen ~30% breder, vult A4 liggend) en lettertype Arial (Excel + dashboard-voorbeeld)
</commit_message>
<xml_diff>
--- a/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
+++ b/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
@@ -31,87 +31,87 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001C1C1E"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="006B6B70"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001B52C4"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001B52C4"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001C1C1E"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="006B6B70"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="001C1C1E"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001C1C1E"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00C2410C"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00C2410C"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="001C1C1E"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="006B6B70"/>
       <sz val="8"/>
@@ -770,22 +770,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="7.2" customWidth="1" min="5" max="5"/>
-    <col width="7.2" customWidth="1" min="6" max="6"/>
-    <col width="7.2" customWidth="1" min="7" max="7"/>
-    <col width="7.2" customWidth="1" min="8" max="8"/>
-    <col width="7.2" customWidth="1" min="9" max="9"/>
-    <col width="7.2" customWidth="1" min="10" max="10"/>
-    <col width="7.2" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="1.5" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9.5" customWidth="1" min="5" max="5"/>
+    <col width="9.5" customWidth="1" min="6" max="6"/>
+    <col width="9.5" customWidth="1" min="7" max="7"/>
+    <col width="9.5" customWidth="1" min="8" max="8"/>
+    <col width="9.5" customWidth="1" min="9" max="9"/>
+    <col width="9.5" customWidth="1" min="10" max="10"/>
+    <col width="9.5" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="2" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="10" customHeight="1"/>

</xml_diff>

<commit_message>
Q4S-Timesheet: onderste blokken uitgelijnd op het raster — klanthandtekening exact onder Kilometers, Akkoord klant even hoog als Medewerker en handtekening (Excel + voorbeeld)
</commit_message>
<xml_diff>
--- a/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
+++ b/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
@@ -1890,6 +1890,12 @@
       <c r="C47" s="16" t="n"/>
       <c r="D47" s="16" t="n"/>
       <c r="E47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="16" t="n"/>
+      <c r="J47" s="16" t="n"/>
+      <c r="K47" s="16" t="n"/>
+      <c r="L47" s="16" t="n"/>
       <c r="N47" s="16" t="n"/>
       <c r="O47" s="16" t="n"/>
       <c r="P47" s="16" t="n"/>
@@ -1922,11 +1928,11 @@
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="B18:D18"/>
-    <mergeCell ref="G46:H46"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="G43:H43"/>
     <mergeCell ref="B49:Q49"/>
     <mergeCell ref="I44:L44"/>
+    <mergeCell ref="I46:L47"/>
     <mergeCell ref="C35:L36"/>
     <mergeCell ref="C29:L30"/>
     <mergeCell ref="N10:Q10"/>
@@ -1947,9 +1953,9 @@
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="N40:P40"/>
     <mergeCell ref="N17:N19"/>
+    <mergeCell ref="G46:H47"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="C44:E44"/>
-    <mergeCell ref="I46:L46"/>
     <mergeCell ref="N29:N31"/>
     <mergeCell ref="C27:L28"/>
   </mergeCells>

</xml_diff>

<commit_message>
Q4S-Timesheet: bedrijfsregels onderaan (adres, website, info@q4s.nl / tel, KvK, BTW, IBAN) in Excel + voorbeeld; voorbeeld iets compacter zodat alles op één A4 liggend past
</commit_message>
<xml_diff>
--- a/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
+++ b/public/templates/urenstaat/Q4S-Timesheet-EN.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4S-Timesheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Q4S-Timesheet'!$B$2:$Q$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Q4S-Timesheet'!$B$2:$Q$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
     <numFmt numFmtId="165" formatCode="DD-MM"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,6 +115,12 @@
       <i val="1"/>
       <color rgb="006B6B70"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="001C1C1E"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -251,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -370,6 +376,13 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -766,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:Q49"/>
+  <dimension ref="B2:Q52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1909,8 +1922,38 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51">
+      <c r="B51" s="43" t="inlineStr">
+        <is>
+          <t>Q4S B.V., Arnhemseweg 12, 2994LA, Barendrecht, the Netherlands, www.q4s.nl, email: info@q4s.nl</t>
+        </is>
+      </c>
+      <c r="C51" s="44" t="n"/>
+      <c r="D51" s="44" t="n"/>
+      <c r="E51" s="44" t="n"/>
+      <c r="F51" s="44" t="n"/>
+      <c r="G51" s="44" t="n"/>
+      <c r="H51" s="44" t="n"/>
+      <c r="I51" s="44" t="n"/>
+      <c r="J51" s="44" t="n"/>
+      <c r="K51" s="44" t="n"/>
+      <c r="L51" s="44" t="n"/>
+      <c r="M51" s="44" t="n"/>
+      <c r="N51" s="44" t="n"/>
+      <c r="O51" s="44" t="n"/>
+      <c r="P51" s="44" t="n"/>
+      <c r="Q51" s="44" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>Tel: +31(0) 857826818, KvK:69073287, Btw: NL857718137B01, IBAN: NL96INGB0007873625</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="49">
     <mergeCell ref="C43:E43"/>
     <mergeCell ref="N37:N39"/>
     <mergeCell ref="N13:N15"/>
@@ -1936,6 +1979,7 @@
     <mergeCell ref="C35:L36"/>
     <mergeCell ref="C29:L30"/>
     <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="B52:Q52"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="N21:N23"/>
     <mergeCell ref="B20:D20"/>
@@ -1954,6 +1998,7 @@
     <mergeCell ref="N40:P40"/>
     <mergeCell ref="N17:N19"/>
     <mergeCell ref="G46:H47"/>
+    <mergeCell ref="B51:Q51"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="C44:E44"/>
     <mergeCell ref="N29:N31"/>
@@ -1968,14 +2013,6 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;7 &amp;K8A8A90Q4S B.V. · Arnhemseweg 12, 2994LA Barendrecht · www.q4s.nl · admin@q4s.nl · KvK 69073287</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>